<commit_message>
Who Comes Back to Court?: remove repeated lines
Maintainer-picked: a new intro headline so it no longer echoes the
title (thumbnail retaken), the Meehl paragraph stops restating the
research claim the score line carries, the Teaching Prompt drops its
second "studying" clause and the "tenth file" line, the Dawes note
drops its "tired, bored, or charmed" ending, and one case note stops
saying "the gut" twice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191t4cG3m6aQycW3EiNAUvs
</commit_message>
<xml_diff>
--- a/gut/data/gut_cases.xlsx
+++ b/gut/data/gut_cases.xlsx
@@ -505,7 +505,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>The one file where everything points the same way. Easy for the gut, easy for the rule. Cases like this teach the gut false confidence.</t>
+          <t>The one file where everything points the same way. Easy for the gut, easy for the rule, and cases like this are where false confidence comes from.</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Even crude models with unit weights tend to outperform the experts who built them, because they never get tired, bored, or charmed.</t>
+          <t>Even crude models with unit weights tend to outperform the experts who built them.</t>
         </is>
       </c>
     </row>

</xml_diff>